<commit_message>
Painel para ecrã largo; linha fixa só nos resumos largos, sem atravessar texto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exemplo/exemplo-transformacao.xlsx
+++ b/docs/exemplo/exemplo-transformacao.xlsx
@@ -38,7 +38,7 @@
     <numFmt numFmtId="177" formatCode="0.0 &quot;cm&quot;"/>
     <numFmt numFmtId="178" formatCode="+0.0 &quot;cm&quot;;-0.0 &quot;cm&quot;;0.0 &quot;cm&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,19 +73,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="0052616B"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00263238"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="0052616B"/>
-      <sz val="8"/>
+      <sz val="24"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -228,12 +222,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -263,12 +257,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -348,7 +342,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2288,21 +2282,21 @@
   <dimension ref="A1:O99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="2" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="2" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="2" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="3" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2313,12 +2307,12 @@
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2">
-        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;YEAR(MAX('Medições Corporais'!$A$4:$A$147))&amp;" às "&amp;RIGHT("0"&amp;HOUR(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 12:16"</f>
+        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;YEAR(MAX('Medições Corporais'!$A$4:$A$147))&amp;" às "&amp;RIGHT("0"&amp;HOUR(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 12:43"</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="17" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Último peso</t>
@@ -2348,7 +2342,7 @@
       <c r="N4" s="7" t="n"/>
       <c r="O4" s="8" t="n"/>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="17" customHeight="1">
       <c r="A5" s="9">
         <f>INDEX('Medições Corporais'!$B$4:$B$147,MATCH(MAX('Medições Corporais'!$A$4:$A$147),'Medições Corporais'!$A$4:$A$147,0))</f>
         <v/>
@@ -2374,7 +2368,7 @@
       <c r="N5" s="13" t="n"/>
       <c r="O5" s="14" t="n"/>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="17" customHeight="1">
       <c r="A6" s="16" t="n"/>
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="11" t="n"/>
@@ -2388,7 +2382,7 @@
       <c r="N6" s="13" t="n"/>
       <c r="O6" s="14" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="17" customHeight="1">
       <c r="A7" s="16" t="n"/>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="11" t="n"/>
@@ -2402,7 +2396,7 @@
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="14" t="n"/>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="17" customHeight="1">
       <c r="A8" s="18">
         <f>"leitura mais recente"</f>
         <v/>
@@ -2429,7 +2423,7 @@
       <c r="O8" s="23" t="n"/>
     </row>
     <row r="9" ht="8" customHeight="1"/>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="17" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Gordura (média 7 dias)</t>
@@ -2459,7 +2453,7 @@
       <c r="N10" s="7" t="n"/>
       <c r="O10" s="8" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="17" customHeight="1">
       <c r="A11" s="30">
         <f>AVERAGEIFS('Medições Corporais'!$D$4:$D$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)</f>
         <v/>
@@ -2485,7 +2479,7 @@
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="14" t="n"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="17" customHeight="1">
       <c r="A12" s="37" t="n"/>
       <c r="B12" s="31" t="n"/>
       <c r="C12" s="32" t="n"/>
@@ -2499,7 +2493,7 @@
       <c r="N12" s="13" t="n"/>
       <c r="O12" s="14" t="n"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="17" customHeight="1">
       <c r="A13" s="37" t="n"/>
       <c r="B13" s="31" t="n"/>
       <c r="C13" s="32" t="n"/>
@@ -2513,7 +2507,7 @@
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="14" t="n"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="17" customHeight="1">
       <c r="A14" s="39">
         <f>"estimativa da balança"</f>
         <v/>
@@ -2540,7 +2534,7 @@
       <c r="O14" s="23" t="n"/>
     </row>
     <row r="15" ht="8" customHeight="1"/>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="17" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
           <t>Última cintura</t>
@@ -2570,7 +2564,7 @@
       <c r="N16" s="7" t="n"/>
       <c r="O16" s="8" t="n"/>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="17" customHeight="1">
       <c r="A17" s="45">
         <f>IF(COUNT('Medidas Manuais'!$C$4:$C$25)=0,"",SUMIFS('Medidas Manuais'!$C$4:$C$25,'Medidas Manuais'!$B$4:$B$25,_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")))</f>
         <v/>
@@ -2596,7 +2590,7 @@
       <c r="N17" s="13" t="n"/>
       <c r="O17" s="14" t="n"/>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="17" customHeight="1">
       <c r="A18" s="37" t="n"/>
       <c r="B18" s="31" t="n"/>
       <c r="C18" s="32" t="n"/>
@@ -2610,7 +2604,7 @@
       <c r="N18" s="13" t="n"/>
       <c r="O18" s="14" t="n"/>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="17" customHeight="1">
       <c r="A19" s="37" t="n"/>
       <c r="B19" s="31" t="n"/>
       <c r="C19" s="32" t="n"/>
@@ -2624,7 +2618,7 @@
       <c r="N19" s="13" t="n"/>
       <c r="O19" s="14" t="n"/>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="17" customHeight="1">
       <c r="A20" s="39">
         <f>IF(COUNT('Medidas Manuais'!$C$4:$C$25)=0,"","medida em "&amp;RIGHT("0"&amp;DAY(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")),2)&amp;"/"&amp;YEAR(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")))</f>
         <v/>
@@ -2740,16 +2734,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Resumo mensal</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="49" t="inlineStr">
-        <is>
-          <t>Atualizado em 11/10/2026 12:16</t>
+      <c r="B2" s="49" t="inlineStr">
+        <is>
+          <t>Atualizado em 11/10/2026 12:43</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3353,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="48" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>Médias aritméticas das leituras aceites do período (não médias diárias). Variação = média do período menos a do período anterior; gordura em pontos percentuais. 'Período parcial' = começa antes do início da transformação ou termina depois da última leitura. Cintura e pescoço: média das medições manuais com data nesse mês.</t>
         </is>
@@ -3367,9 +3361,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="A11:N11"/>
-    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="B11:O11"/>
+    <mergeCell ref="B1:U1"/>
+    <mergeCell ref="B2:U2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:U9">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -3425,16 +3419,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Resumo semanal (domingo a sábado)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="49" t="inlineStr">
-        <is>
-          <t>Atualizado em 11/10/2026 12:16</t>
+      <c r="B2" s="49" t="inlineStr">
+        <is>
+          <t>Atualizado em 11/10/2026 12:43</t>
         </is>
       </c>
     </row>
@@ -5509,7 +5503,7 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="48" t="inlineStr">
+      <c r="B27" s="48" t="inlineStr">
         <is>
           <t>Médias aritméticas das leituras aceites do período (não médias diárias). Variação = média do período menos a do período anterior; gordura em pontos percentuais. 'Período parcial' = começa antes do início da transformação ou termina depois da última leitura. Cintura: diferença face à medição anterior disponível.</t>
         </is>
@@ -5517,9 +5511,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:V2"/>
-    <mergeCell ref="A27:N27"/>
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="B27:O27"/>
+    <mergeCell ref="B1:V1"/>
+    <mergeCell ref="B2:V2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:V25">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -6293,7 +6287,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>144 leituras aceites · Atualizado em 11/10/2026 12:16 · fórmulas: massa gorda e médias móveis de 7 dias</t>
+          <t>144 leituras aceites · Atualizado em 11/10/2026 12:43 · fórmulas: massa gorda e médias móveis de 7 dias</t>
         </is>
       </c>
     </row>
@@ -14778,7 +14772,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:16</t>
+          <t>Atualizado em 11/10/2026 12:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel: margens laterais com a largura dos espaços entre cartões
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exemplo/exemplo-transformacao.xlsx
+++ b/docs/exemplo/exemplo-transformacao.xlsx
@@ -1750,13 +1750,13 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
-      <col>0</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <to>
-      <col>15</col>
+      <col>16</col>
       <colOff>0</colOff>
       <row>40</row>
       <rowOff>0</rowOff>
@@ -1777,13 +1777,13 @@
   </twoCellAnchor>
   <twoCellAnchor editAs="oneCell">
     <from>
-      <col>0</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>41</row>
       <rowOff>0</rowOff>
     </from>
     <to>
-      <col>15</col>
+      <col>16</col>
       <colOff>0</colOff>
       <row>59</row>
       <rowOff>0</rowOff>
@@ -1804,13 +1804,13 @@
   </twoCellAnchor>
   <twoCellAnchor editAs="oneCell">
     <from>
-      <col>0</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>60</row>
       <rowOff>0</rowOff>
     </from>
     <to>
-      <col>15</col>
+      <col>16</col>
       <colOff>0</colOff>
       <row>78</row>
       <rowOff>0</rowOff>
@@ -1831,13 +1831,13 @@
   </twoCellAnchor>
   <twoCellAnchor editAs="oneCell">
     <from>
-      <col>0</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>79</row>
       <rowOff>0</rowOff>
     </from>
     <to>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>97</row>
       <rowOff>0</rowOff>
@@ -1858,13 +1858,13 @@
   </twoCellAnchor>
   <twoCellAnchor editAs="oneCell">
     <from>
-      <col>8</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>79</row>
       <rowOff>0</rowOff>
     </from>
     <to>
-      <col>15</col>
+      <col>16</col>
       <colOff>0</colOff>
       <row>97</row>
       <rowOff>0</rowOff>
@@ -2279,374 +2279,376 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O99"/>
+  <dimension ref="B1:P99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="3" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="3" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="3" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="15.5" customWidth="1" min="2" max="2"/>
+    <col width="15.5" customWidth="1" min="3" max="3"/>
+    <col width="15.5" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="15.5" customWidth="1" min="6" max="6"/>
+    <col width="15.5" customWidth="1" min="7" max="7"/>
+    <col width="15.5" customWidth="1" min="8" max="8"/>
+    <col width="3" customWidth="1" min="9" max="9"/>
+    <col width="15.5" customWidth="1" min="10" max="10"/>
+    <col width="15.5" customWidth="1" min="11" max="11"/>
+    <col width="15.5" customWidth="1" min="12" max="12"/>
+    <col width="3" customWidth="1" min="13" max="13"/>
+    <col width="15.5" customWidth="1" min="14" max="14"/>
+    <col width="15.5" customWidth="1" min="15" max="15"/>
+    <col width="15.5" customWidth="1" min="16" max="16"/>
+    <col width="3" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1">
+      <c r="B1" s="1">
         <f>"Transformação corporal  ·  04/01/2026 a "&amp;RIGHT("0"&amp;DAY(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;YEAR(MAX('Medições Corporais'!$A$4:$A$147))</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2">
-        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;YEAR(MAX('Medições Corporais'!$A$4:$A$147))&amp;" às "&amp;RIGHT("0"&amp;HOUR(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 12:43"</f>
+      <c r="B2" s="2">
+        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;YEAR(MAX('Medições Corporais'!$A$4:$A$147))&amp;" às "&amp;RIGHT("0"&amp;HOUR(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 12:46"</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Último peso</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Peso (média 7 dias)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Peso desde o início</t>
         </is>
       </c>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="8" t="n"/>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="K4" s="7" t="n"/>
+      <c r="L4" s="8" t="n"/>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Ritmo recente</t>
         </is>
       </c>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="8" t="n"/>
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="8" t="n"/>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="9">
+      <c r="B5" s="9">
         <f>INDEX('Medições Corporais'!$B$4:$B$147,MATCH(MAX('Medições Corporais'!$A$4:$A$147),'Medições Corporais'!$A$4:$A$147,0))</f>
         <v/>
       </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="11" t="n"/>
-      <c r="E5" s="9">
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="F5" s="9">
         <f>AVERAGEIFS('Medições Corporais'!$B$4:$B$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)</f>
         <v/>
       </c>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="11" t="n"/>
-      <c r="I5" s="12">
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="11" t="n"/>
+      <c r="J5" s="12">
         <f>AVERAGEIFS('Medições Corporais'!$B$4:$B$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)-AVERAGEIFS('Medições Corporais'!$B$4:$B$147,'Medições Corporais'!$A$4:$A$147,"&lt;"&amp;MIN('Medições Corporais'!$A$4:$A$147)+7)</f>
         <v/>
       </c>
-      <c r="J5" s="13" t="n"/>
-      <c r="K5" s="14" t="n"/>
-      <c r="M5" s="15">
+      <c r="K5" s="13" t="n"/>
+      <c r="L5" s="14" t="n"/>
+      <c r="N5" s="15">
         <f>IFERROR((AVERAGEIFS('Medições Corporais'!$B$4:$B$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)-AVERAGEIFS('Medições Corporais'!$B$4:$B$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-28,'Medições Corporais'!$A$4:$A$147,"&lt;="&amp;MAX('Medições Corporais'!$A$4:$A$147)-21))/3,"")</f>
         <v/>
       </c>
-      <c r="N5" s="13" t="n"/>
-      <c r="O5" s="14" t="n"/>
+      <c r="O5" s="13" t="n"/>
+      <c r="P5" s="14" t="n"/>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="11" t="n"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="13" t="n"/>
-      <c r="K6" s="14" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="13" t="n"/>
-      <c r="O6" s="14" t="n"/>
+      <c r="B6" s="16" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="11" t="n"/>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="13" t="n"/>
+      <c r="L6" s="14" t="n"/>
+      <c r="N6" s="17" t="n"/>
+      <c r="O6" s="13" t="n"/>
+      <c r="P6" s="14" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="16" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="11" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="13" t="n"/>
-      <c r="K7" s="14" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="13" t="n"/>
-      <c r="O7" s="14" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="13" t="n"/>
+      <c r="L7" s="14" t="n"/>
+      <c r="N7" s="17" t="n"/>
+      <c r="O7" s="13" t="n"/>
+      <c r="P7" s="14" t="n"/>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="18">
+      <c r="B8" s="18">
         <f>"leitura mais recente"</f>
         <v/>
       </c>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="E8" s="18">
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="20" t="n"/>
+      <c r="F8" s="18">
         <f>"últimos 7 dias"</f>
         <v/>
       </c>
-      <c r="F8" s="19" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="I8" s="21">
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="20" t="n"/>
+      <c r="J8" s="21">
         <f>"média 7 dias: atual − inicial"</f>
         <v/>
       </c>
-      <c r="J8" s="22" t="n"/>
-      <c r="K8" s="23" t="n"/>
-      <c r="M8" s="21">
+      <c r="K8" s="22" t="n"/>
+      <c r="L8" s="23" t="n"/>
+      <c r="N8" s="21">
         <f>"últimas 4 semanas"</f>
         <v/>
       </c>
-      <c r="N8" s="22" t="n"/>
-      <c r="O8" s="23" t="n"/>
+      <c r="O8" s="22" t="n"/>
+      <c r="P8" s="23" t="n"/>
     </row>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Gordura (média 7 dias)</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n"/>
-      <c r="C10" s="26" t="n"/>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="C10" s="25" t="n"/>
+      <c r="D10" s="26" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Gordura desde o início</t>
         </is>
       </c>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="I10" s="27" t="inlineStr">
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="J10" s="27" t="inlineStr">
         <is>
           <t>Músculo (média 7 dias)</t>
         </is>
       </c>
-      <c r="J10" s="28" t="n"/>
-      <c r="K10" s="29" t="n"/>
-      <c r="M10" s="6" t="inlineStr">
+      <c r="K10" s="28" t="n"/>
+      <c r="L10" s="29" t="n"/>
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>Músculo desde o início</t>
         </is>
       </c>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="8" t="n"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="8" t="n"/>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="30">
+      <c r="B11" s="30">
         <f>AVERAGEIFS('Medições Corporais'!$D$4:$D$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)</f>
         <v/>
       </c>
-      <c r="B11" s="31" t="n"/>
-      <c r="C11" s="32" t="n"/>
-      <c r="E11" s="33">
+      <c r="C11" s="31" t="n"/>
+      <c r="D11" s="32" t="n"/>
+      <c r="F11" s="33">
         <f>AVERAGEIFS('Medições Corporais'!$D$4:$D$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)-AVERAGEIFS('Medições Corporais'!$D$4:$D$147,'Medições Corporais'!$A$4:$A$147,"&lt;"&amp;MIN('Medições Corporais'!$A$4:$A$147)+7)</f>
         <v/>
       </c>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="14" t="n"/>
-      <c r="I11" s="34">
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="14" t="n"/>
+      <c r="J11" s="34">
         <f>AVERAGEIFS('Medições Corporais'!$G$4:$G$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)</f>
         <v/>
       </c>
-      <c r="J11" s="35" t="n"/>
-      <c r="K11" s="36" t="n"/>
-      <c r="M11" s="12">
+      <c r="K11" s="35" t="n"/>
+      <c r="L11" s="36" t="n"/>
+      <c r="N11" s="12">
         <f>AVERAGEIFS('Medições Corporais'!$G$4:$G$147,'Medições Corporais'!$A$4:$A$147,"&gt;"&amp;MAX('Medições Corporais'!$A$4:$A$147)-7)-AVERAGEIFS('Medições Corporais'!$G$4:$G$147,'Medições Corporais'!$A$4:$A$147,"&lt;"&amp;MIN('Medições Corporais'!$A$4:$A$147)+7)</f>
         <v/>
       </c>
-      <c r="N11" s="13" t="n"/>
-      <c r="O11" s="14" t="n"/>
+      <c r="O11" s="13" t="n"/>
+      <c r="P11" s="14" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="37" t="n"/>
-      <c r="B12" s="31" t="n"/>
-      <c r="C12" s="32" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="14" t="n"/>
-      <c r="I12" s="38" t="n"/>
-      <c r="J12" s="35" t="n"/>
-      <c r="K12" s="36" t="n"/>
-      <c r="M12" s="17" t="n"/>
-      <c r="N12" s="13" t="n"/>
-      <c r="O12" s="14" t="n"/>
+      <c r="B12" s="37" t="n"/>
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="32" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="14" t="n"/>
+      <c r="J12" s="38" t="n"/>
+      <c r="K12" s="35" t="n"/>
+      <c r="L12" s="36" t="n"/>
+      <c r="N12" s="17" t="n"/>
+      <c r="O12" s="13" t="n"/>
+      <c r="P12" s="14" t="n"/>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="37" t="n"/>
-      <c r="B13" s="31" t="n"/>
-      <c r="C13" s="32" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="I13" s="38" t="n"/>
-      <c r="J13" s="35" t="n"/>
-      <c r="K13" s="36" t="n"/>
-      <c r="M13" s="17" t="n"/>
-      <c r="N13" s="13" t="n"/>
-      <c r="O13" s="14" t="n"/>
+      <c r="B13" s="37" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="14" t="n"/>
+      <c r="J13" s="38" t="n"/>
+      <c r="K13" s="35" t="n"/>
+      <c r="L13" s="36" t="n"/>
+      <c r="N13" s="17" t="n"/>
+      <c r="O13" s="13" t="n"/>
+      <c r="P13" s="14" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="39">
+      <c r="B14" s="39">
         <f>"estimativa da balança"</f>
         <v/>
       </c>
-      <c r="B14" s="40" t="n"/>
-      <c r="C14" s="41" t="n"/>
-      <c r="E14" s="21">
+      <c r="C14" s="40" t="n"/>
+      <c r="D14" s="41" t="n"/>
+      <c r="F14" s="21">
         <f>"pontos percentuais"</f>
         <v/>
       </c>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="23" t="n"/>
-      <c r="I14" s="42">
+      <c r="G14" s="22" t="n"/>
+      <c r="H14" s="23" t="n"/>
+      <c r="J14" s="42">
         <f>"estimativa da balança"</f>
         <v/>
       </c>
-      <c r="J14" s="43" t="n"/>
-      <c r="K14" s="44" t="n"/>
-      <c r="M14" s="21">
+      <c r="K14" s="43" t="n"/>
+      <c r="L14" s="44" t="n"/>
+      <c r="N14" s="21">
         <f>"média 7 dias: atual − inicial"</f>
         <v/>
       </c>
-      <c r="N14" s="22" t="n"/>
-      <c r="O14" s="23" t="n"/>
+      <c r="O14" s="22" t="n"/>
+      <c r="P14" s="23" t="n"/>
     </row>
     <row r="15" ht="8" customHeight="1"/>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>Última cintura</t>
         </is>
       </c>
-      <c r="B16" s="25" t="n"/>
-      <c r="C16" s="26" t="n"/>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="C16" s="25" t="n"/>
+      <c r="D16" s="26" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Cintura desde o início</t>
         </is>
       </c>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>Último pescoço</t>
         </is>
       </c>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="5" t="n"/>
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>Pescoço desde o início</t>
         </is>
       </c>
-      <c r="N16" s="7" t="n"/>
-      <c r="O16" s="8" t="n"/>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="8" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="45">
+      <c r="B17" s="45">
         <f>IF(COUNT('Medidas Manuais'!$C$4:$C$25)=0,"",SUMIFS('Medidas Manuais'!$C$4:$C$25,'Medidas Manuais'!$B$4:$B$25,_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")))</f>
         <v/>
       </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="32" t="n"/>
-      <c r="E17" s="46">
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="32" t="n"/>
+      <c r="F17" s="46">
         <f>IF(COUNT('Medidas Manuais'!$C$4:$C$25)&lt;2,"",SUMIFS('Medidas Manuais'!$C$4:$C$25,'Medidas Manuais'!$B$4:$B$25,_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0"))-SUMIFS('Medidas Manuais'!$C$4:$C$25,'Medidas Manuais'!$B$4:$B$25,_xlfn.MINIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")))</f>
         <v/>
       </c>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="I17" s="47">
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="14" t="n"/>
+      <c r="J17" s="47">
         <f>IF(COUNT('Medidas Manuais'!$E$4:$E$25)=0,"",SUMIFS('Medidas Manuais'!$E$4:$E$25,'Medidas Manuais'!$B$4:$B$25,_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$E$4:$E$25,"&gt;0")))</f>
         <v/>
       </c>
-      <c r="J17" s="10" t="n"/>
-      <c r="K17" s="11" t="n"/>
-      <c r="M17" s="46">
+      <c r="K17" s="10" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="N17" s="46">
         <f>IF(COUNT('Medidas Manuais'!$E$4:$E$25)&lt;2,"",SUMIFS('Medidas Manuais'!$E$4:$E$25,'Medidas Manuais'!$B$4:$B$25,_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$E$4:$E$25,"&gt;0"))-SUMIFS('Medidas Manuais'!$E$4:$E$25,'Medidas Manuais'!$B$4:$B$25,_xlfn.MINIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$E$4:$E$25,"&gt;0")))</f>
         <v/>
       </c>
-      <c r="N17" s="13" t="n"/>
-      <c r="O17" s="14" t="n"/>
+      <c r="O17" s="13" t="n"/>
+      <c r="P17" s="14" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="37" t="n"/>
-      <c r="B18" s="31" t="n"/>
-      <c r="C18" s="32" t="n"/>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="14" t="n"/>
-      <c r="I18" s="16" t="n"/>
-      <c r="J18" s="10" t="n"/>
-      <c r="K18" s="11" t="n"/>
-      <c r="M18" s="17" t="n"/>
-      <c r="N18" s="13" t="n"/>
-      <c r="O18" s="14" t="n"/>
+      <c r="B18" s="37" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="32" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="n"/>
+      <c r="J18" s="16" t="n"/>
+      <c r="K18" s="10" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="N18" s="17" t="n"/>
+      <c r="O18" s="13" t="n"/>
+      <c r="P18" s="14" t="n"/>
     </row>
     <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="37" t="n"/>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="32" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="I19" s="16" t="n"/>
-      <c r="J19" s="10" t="n"/>
-      <c r="K19" s="11" t="n"/>
-      <c r="M19" s="17" t="n"/>
-      <c r="N19" s="13" t="n"/>
-      <c r="O19" s="14" t="n"/>
+      <c r="B19" s="37" t="n"/>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="14" t="n"/>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="11" t="n"/>
+      <c r="N19" s="17" t="n"/>
+      <c r="O19" s="13" t="n"/>
+      <c r="P19" s="14" t="n"/>
     </row>
     <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="39">
+      <c r="B20" s="39">
         <f>IF(COUNT('Medidas Manuais'!$C$4:$C$25)=0,"","medida em "&amp;RIGHT("0"&amp;DAY(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")),2)&amp;"/"&amp;YEAR(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$C$4:$C$25,"&gt;0")))</f>
         <v/>
       </c>
-      <c r="B20" s="40" t="n"/>
-      <c r="C20" s="41" t="n"/>
-      <c r="E20" s="21">
+      <c r="C20" s="40" t="n"/>
+      <c r="D20" s="41" t="n"/>
+      <c r="F20" s="21">
         <f>"última − primeira medição"</f>
         <v/>
       </c>
-      <c r="F20" s="22" t="n"/>
-      <c r="G20" s="23" t="n"/>
-      <c r="I20" s="18">
+      <c r="G20" s="22" t="n"/>
+      <c r="H20" s="23" t="n"/>
+      <c r="J20" s="18">
         <f>IF(COUNT('Medidas Manuais'!$E$4:$E$25)=0,"","medido em "&amp;RIGHT("0"&amp;DAY(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$E$4:$E$25,"&gt;0")),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$E$4:$E$25,"&gt;0")),2)&amp;"/"&amp;YEAR(_xlfn.MAXIFS('Medidas Manuais'!$B$4:$B$25,'Medidas Manuais'!$E$4:$E$25,"&gt;0")))</f>
         <v/>
       </c>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="20" t="n"/>
-      <c r="M20" s="21">
+      <c r="K20" s="19" t="n"/>
+      <c r="L20" s="20" t="n"/>
+      <c r="N20" s="21">
         <f>"última − primeira medição"</f>
         <v/>
       </c>
-      <c r="N20" s="22" t="n"/>
-      <c r="O20" s="23" t="n"/>
+      <c r="O20" s="22" t="n"/>
+      <c r="P20" s="23" t="n"/>
     </row>
     <row r="21" ht="8" customHeight="1"/>
     <row r="99" ht="30" customHeight="1">
-      <c r="A99" s="48" t="inlineStr">
+      <c r="B99" s="48" t="inlineStr">
         <is>
           <t>Gráficos de peso, gordura e músculo: pontos = leituras; linha = média móvel de 7 dias. Cintura e pescoço: pontos = medições reais; tracejado = semanas sem medição (só visual, sem valores inventados). As escalas e os tracejados são recalculados em cada atualização.</t>
         </is>
@@ -2654,44 +2656,44 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="I11:K13"/>
-    <mergeCell ref="E5:G7"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="M11:O13"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="A99:O99"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="I5:K7"/>
-    <mergeCell ref="I17:K19"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="A17:C19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="E11:G13"/>
-    <mergeCell ref="A5:C7"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="M4:O4"/>
-    <mergeCell ref="M17:O19"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="M5:O7"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="E17:G19"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="A11:C13"/>
-    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="F5:H7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B1:P1"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N5:P7"/>
+    <mergeCell ref="B17:D19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="J11:L13"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="F17:H19"/>
+    <mergeCell ref="B99:P99"/>
+    <mergeCell ref="N17:P19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="B5:D7"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="N11:P13"/>
+    <mergeCell ref="F11:H13"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="J5:L7"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="J17:L19"/>
+    <mergeCell ref="B11:D13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
@@ -2743,7 +2745,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:43</t>
+          <t>Atualizado em 11/10/2026 12:46</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3430,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:43</t>
+          <t>Atualizado em 11/10/2026 12:46</t>
         </is>
       </c>
     </row>
@@ -6287,7 +6289,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>144 leituras aceites · Atualizado em 11/10/2026 12:43 · fórmulas: massa gorda e médias móveis de 7 dias</t>
+          <t>144 leituras aceites · Atualizado em 11/10/2026 12:46 · fórmulas: massa gorda e médias móveis de 7 dias</t>
         </is>
       </c>
     </row>
@@ -14772,7 +14774,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:43</t>
+          <t>Atualizado em 11/10/2026 12:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel: espaçamento único em margens, cartões e gráficos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exemplo/exemplo-transformacao.xlsx
+++ b/docs/exemplo/exemplo-transformacao.xlsx
@@ -21,22 +21,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="15">
+  <numFmts count="16">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="169" formatCode="+0.0;-0.0;0.0"/>
-    <numFmt numFmtId="170" formatCode="+0.00;-0.00;0.00"/>
-    <numFmt numFmtId="171" formatCode="[$-816]mmmm yyyy"/>
-    <numFmt numFmtId="172" formatCode="0.00 &quot;kg&quot;"/>
-    <numFmt numFmtId="173" formatCode="+0.00 &quot;kg&quot;;-0.00 &quot;kg&quot;;0.00 &quot;kg&quot;"/>
-    <numFmt numFmtId="174" formatCode="+0.00 &quot;kg/sem.&quot;;-0.00 &quot;kg/sem.&quot;;0.00 &quot;kg/sem.&quot;"/>
-    <numFmt numFmtId="175" formatCode="0.0 &quot;%&quot;"/>
-    <numFmt numFmtId="176" formatCode="+0.0 &quot;pp&quot;;-0.0 &quot;pp&quot;;0.0 &quot;pp&quot;"/>
-    <numFmt numFmtId="177" formatCode="0.0 &quot;cm&quot;"/>
-    <numFmt numFmtId="178" formatCode="+0.0 &quot;cm&quot;;-0.0 &quot;cm&quot;;0.0 &quot;cm&quot;"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yyyy hh:mm:ss"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="170" formatCode="+0.0;-0.0;0.0"/>
+    <numFmt numFmtId="171" formatCode="+0.00;-0.00;0.00"/>
+    <numFmt numFmtId="172" formatCode="[$-816]mmmm yyyy"/>
+    <numFmt numFmtId="173" formatCode="0.00 &quot;kg&quot;"/>
+    <numFmt numFmtId="174" formatCode="+0.00 &quot;kg&quot;;-0.00 &quot;kg&quot;;0.00 &quot;kg&quot;"/>
+    <numFmt numFmtId="175" formatCode="+0.00 &quot;kg/sem.&quot;;-0.00 &quot;kg/sem.&quot;;0.00 &quot;kg/sem.&quot;"/>
+    <numFmt numFmtId="176" formatCode="0.0 &quot;%&quot;"/>
+    <numFmt numFmtId="177" formatCode="+0.0 &quot;pp&quot;;-0.0 &quot;pp&quot;;0.0 &quot;pp&quot;"/>
+    <numFmt numFmtId="178" formatCode="0.0 &quot;cm&quot;"/>
+    <numFmt numFmtId="179" formatCode="+0.0 &quot;cm&quot;;-0.0 &quot;cm&quot;;0.0 &quot;cm&quot;"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -191,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -207,17 +208,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="172" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="174" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="174" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -242,15 +243,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="175" fontId="6" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="6" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="177" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="6" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -267,13 +268,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="6" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="6" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="179" fontId="6" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -294,7 +295,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -309,13 +310,13 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -337,6 +338,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1752,13 +1756,13 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>16</col>
       <colOff>0</colOff>
-      <row>40</row>
+      <row>39</row>
       <rowOff>0</rowOff>
     </to>
     <graphicFrame>
@@ -1779,13 +1783,13 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>41</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>16</col>
       <colOff>0</colOff>
-      <row>59</row>
+      <row>58</row>
       <rowOff>0</rowOff>
     </to>
     <graphicFrame>
@@ -1806,13 +1810,13 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>60</row>
+      <row>59</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>16</col>
       <colOff>0</colOff>
-      <row>78</row>
+      <row>77</row>
       <rowOff>0</rowOff>
     </to>
     <graphicFrame>
@@ -1833,13 +1837,13 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>79</row>
+      <row>78</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>8</col>
       <colOff>0</colOff>
-      <row>97</row>
+      <row>96</row>
       <rowOff>0</rowOff>
     </to>
     <graphicFrame>
@@ -1860,13 +1864,13 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>79</row>
+      <row>78</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>16</col>
       <colOff>0</colOff>
-      <row>97</row>
+      <row>96</row>
       <rowOff>0</rowOff>
     </to>
     <graphicFrame>
@@ -1964,9 +1968,9 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCorpo" displayName="tblCorpo" ref="A3:Q147" headerRowCount="1">
-  <autoFilter ref="A3:Q147"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCorpo" displayName="tblCorpo" ref="A3:R147" headerRowCount="1">
+  <autoFilter ref="A3:R147"/>
+  <tableColumns count="18">
     <tableColumn id="1" name="Data/hora"/>
     <tableColumn id="2" name="Peso (kg)"/>
     <tableColumn id="3" name="IMC"/>
@@ -1984,6 +1988,7 @@
     <tableColumn id="15" name="Gordura, média 7 dias (%)"/>
     <tableColumn id="16" name="Músculo, média 7 dias (kg)"/>
     <tableColumn id="17" name="Dia"/>
+    <tableColumn id="18" name="Instante UTC"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -2279,25 +2284,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P99"/>
+  <dimension ref="B1:P98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="15.5" customWidth="1" min="2" max="2"/>
-    <col width="15.5" customWidth="1" min="3" max="3"/>
-    <col width="15.5" customWidth="1" min="4" max="4"/>
+    <col width="15.9" customWidth="1" min="2" max="2"/>
+    <col width="15.9" customWidth="1" min="3" max="3"/>
+    <col width="15.9" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
-    <col width="15.5" customWidth="1" min="6" max="6"/>
-    <col width="15.5" customWidth="1" min="7" max="7"/>
-    <col width="15.5" customWidth="1" min="8" max="8"/>
+    <col width="15.9" customWidth="1" min="6" max="6"/>
+    <col width="15.9" customWidth="1" min="7" max="7"/>
+    <col width="15.9" customWidth="1" min="8" max="8"/>
     <col width="3" customWidth="1" min="9" max="9"/>
-    <col width="15.5" customWidth="1" min="10" max="10"/>
-    <col width="15.5" customWidth="1" min="11" max="11"/>
-    <col width="15.5" customWidth="1" min="12" max="12"/>
+    <col width="15.9" customWidth="1" min="10" max="10"/>
+    <col width="15.9" customWidth="1" min="11" max="11"/>
+    <col width="15.9" customWidth="1" min="12" max="12"/>
     <col width="3" customWidth="1" min="13" max="13"/>
-    <col width="15.5" customWidth="1" min="14" max="14"/>
-    <col width="15.5" customWidth="1" min="15" max="15"/>
-    <col width="15.5" customWidth="1" min="16" max="16"/>
+    <col width="15.9" customWidth="1" min="14" max="14"/>
+    <col width="15.9" customWidth="1" min="15" max="15"/>
+    <col width="15.9" customWidth="1" min="16" max="16"/>
     <col width="3" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -2309,11 +2314,11 @@
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="2">
-        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"/"&amp;YEAR(MAX('Medições Corporais'!$A$4:$A$147))&amp;" às "&amp;RIGHT("0"&amp;HOUR(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(MAX('Medições Corporais'!$A$4:$A$147)),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 12:46"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3" ht="8" customHeight="1"/>
+        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"/"&amp;YEAR(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0)))&amp;" às "&amp;RIGHT("0"&amp;HOUR(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 12:56"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="16.2" customHeight="1"/>
     <row r="4" ht="17" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -2346,7 +2351,7 @@
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="B5" s="9">
-        <f>INDEX('Medições Corporais'!$B$4:$B$147,MATCH(MAX('Medições Corporais'!$A$4:$A$147),'Medições Corporais'!$A$4:$A$147,0))</f>
+        <f>INDEX('Medições Corporais'!$B$4:$B$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))</f>
         <v/>
       </c>
       <c r="C5" s="10" t="n"/>
@@ -2424,7 +2429,7 @@
       <c r="O8" s="22" t="n"/>
       <c r="P8" s="23" t="n"/>
     </row>
-    <row r="9" ht="8" customHeight="1"/>
+    <row r="9" ht="16.2" customHeight="1"/>
     <row r="10" ht="17" customHeight="1">
       <c r="B10" s="24" t="inlineStr">
         <is>
@@ -2535,7 +2540,7 @@
       <c r="O14" s="22" t="n"/>
       <c r="P14" s="23" t="n"/>
     </row>
-    <row r="15" ht="8" customHeight="1"/>
+    <row r="15" ht="16.2" customHeight="1"/>
     <row r="16" ht="17" customHeight="1">
       <c r="B16" s="24" t="inlineStr">
         <is>
@@ -2646,9 +2651,13 @@
       <c r="O20" s="22" t="n"/>
       <c r="P20" s="23" t="n"/>
     </row>
-    <row r="21" ht="8" customHeight="1"/>
-    <row r="99" ht="30" customHeight="1">
-      <c r="B99" s="48" t="inlineStr">
+    <row r="21" ht="16.2" customHeight="1"/>
+    <row r="40" ht="16.2" customHeight="1"/>
+    <row r="59" ht="16.2" customHeight="1"/>
+    <row r="78" ht="16.2" customHeight="1"/>
+    <row r="97" ht="16.2" customHeight="1"/>
+    <row r="98" ht="30" customHeight="1">
+      <c r="B98" s="48" t="inlineStr">
         <is>
           <t>Gráficos de peso, gordura e músculo: pontos = leituras; linha = média móvel de 7 dias. Cintura e pescoço: pontos = medições reais; tracejado = semanas sem medição (só visual, sem valores inventados). As escalas e os tracejados são recalculados em cada atualização.</t>
         </is>
@@ -2661,6 +2670,7 @@
     <mergeCell ref="F5:H7"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="N14:P14"/>
+    <mergeCell ref="B98:P98"/>
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="B1:P1"/>
     <mergeCell ref="J4:L4"/>
@@ -2673,7 +2683,6 @@
     <mergeCell ref="J16:L16"/>
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="F17:H19"/>
-    <mergeCell ref="B99:P99"/>
     <mergeCell ref="N17:P19"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="F14:H14"/>
@@ -2745,7 +2754,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:46</t>
+          <t>Atualizado em 11/10/2026 12:56</t>
         </is>
       </c>
     </row>
@@ -3430,7 +3439,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:46</t>
+          <t>Atualizado em 11/10/2026 12:56</t>
         </is>
       </c>
     </row>
@@ -6257,7 +6266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q147"/>
+  <dimension ref="A1:R147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -6277,6 +6286,7 @@
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col hidden="1" width="11" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="19" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -6289,7 +6299,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>144 leituras aceites · Atualizado em 11/10/2026 12:46 · fórmulas: massa gorda e médias móveis de 7 dias</t>
+          <t>144 leituras aceites · Atualizado em 11/10/2026 12:56 · fórmulas: massa gorda e médias móveis de 7 dias</t>
         </is>
       </c>
     </row>
@@ -6377,6 +6387,11 @@
       <c r="Q3" s="50" t="inlineStr">
         <is>
           <t>Dia</t>
+        </is>
+      </c>
+      <c r="R3" s="50" t="inlineStr">
+        <is>
+          <t>Instante UTC</t>
         </is>
       </c>
     </row>
@@ -6437,6 +6452,9 @@
         <f>INT(A4)</f>
         <v/>
       </c>
+      <c r="R4" s="69" t="n">
+        <v>46026.44027777778</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="67" t="n">
@@ -6495,6 +6513,9 @@
         <f>INT(A5)</f>
         <v/>
       </c>
+      <c r="R5" s="69" t="n">
+        <v>46027.29930555556</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="67" t="n">
@@ -6553,6 +6574,9 @@
         <f>INT(A6)</f>
         <v/>
       </c>
+      <c r="R6" s="69" t="n">
+        <v>46028.31666666667</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="67" t="n">
@@ -6611,6 +6635,9 @@
         <f>INT(A7)</f>
         <v/>
       </c>
+      <c r="R7" s="69" t="n">
+        <v>46029.31041666667</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="67" t="n">
@@ -6669,6 +6696,9 @@
         <f>INT(A8)</f>
         <v/>
       </c>
+      <c r="R8" s="69" t="n">
+        <v>46030.29930555556</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="67" t="n">
@@ -6727,6 +6757,9 @@
         <f>INT(A9)</f>
         <v/>
       </c>
+      <c r="R9" s="69" t="n">
+        <v>46031.31458333333</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="67" t="n">
@@ -6785,6 +6818,9 @@
         <f>INT(A10)</f>
         <v/>
       </c>
+      <c r="R10" s="69" t="n">
+        <v>46033.42361111111</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="67" t="n">
@@ -6843,6 +6879,9 @@
         <f>INT(A11)</f>
         <v/>
       </c>
+      <c r="R11" s="69" t="n">
+        <v>46034.29305555556</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="67" t="n">
@@ -6901,6 +6940,9 @@
         <f>INT(A12)</f>
         <v/>
       </c>
+      <c r="R12" s="69" t="n">
+        <v>46035.30625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="67" t="n">
@@ -6959,6 +7001,9 @@
         <f>INT(A13)</f>
         <v/>
       </c>
+      <c r="R13" s="69" t="n">
+        <v>46036.31180555555</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="67" t="n">
@@ -7017,6 +7062,9 @@
         <f>INT(A14)</f>
         <v/>
       </c>
+      <c r="R14" s="69" t="n">
+        <v>46038.30486111111</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="67" t="n">
@@ -7075,6 +7123,9 @@
         <f>INT(A15)</f>
         <v/>
       </c>
+      <c r="R15" s="69" t="n">
+        <v>46039.42916666667</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="67" t="n">
@@ -7133,6 +7184,9 @@
         <f>INT(A16)</f>
         <v/>
       </c>
+      <c r="R16" s="69" t="n">
+        <v>46040.44375</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="67" t="n">
@@ -7191,6 +7245,9 @@
         <f>INT(A17)</f>
         <v/>
       </c>
+      <c r="R17" s="69" t="n">
+        <v>46041.29722222222</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="67" t="n">
@@ -7249,6 +7306,9 @@
         <f>INT(A18)</f>
         <v/>
       </c>
+      <c r="R18" s="69" t="n">
+        <v>46042.30902777778</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="67" t="n">
@@ -7307,6 +7367,9 @@
         <f>INT(A19)</f>
         <v/>
       </c>
+      <c r="R19" s="69" t="n">
+        <v>46043.32986111111</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="67" t="n">
@@ -7365,6 +7428,9 @@
         <f>INT(A20)</f>
         <v/>
       </c>
+      <c r="R20" s="69" t="n">
+        <v>46043.33194444444</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="67" t="n">
@@ -7423,6 +7489,9 @@
         <f>INT(A21)</f>
         <v/>
       </c>
+      <c r="R21" s="69" t="n">
+        <v>46044.30138888889</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="67" t="n">
@@ -7481,6 +7550,9 @@
         <f>INT(A22)</f>
         <v/>
       </c>
+      <c r="R22" s="69" t="n">
+        <v>46045.30138888889</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="67" t="n">
@@ -7539,6 +7611,9 @@
         <f>INT(A23)</f>
         <v/>
       </c>
+      <c r="R23" s="69" t="n">
+        <v>46046.44027777778</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="67" t="n">
@@ -7597,6 +7672,9 @@
         <f>INT(A24)</f>
         <v/>
       </c>
+      <c r="R24" s="69" t="n">
+        <v>46047.44722222222</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="67" t="n">
@@ -7655,6 +7733,9 @@
         <f>INT(A25)</f>
         <v/>
       </c>
+      <c r="R25" s="69" t="n">
+        <v>46048.32986111111</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="67" t="n">
@@ -7713,6 +7794,9 @@
         <f>INT(A26)</f>
         <v/>
       </c>
+      <c r="R26" s="69" t="n">
+        <v>46049.30902777778</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="67" t="n">
@@ -7771,6 +7855,9 @@
         <f>INT(A27)</f>
         <v/>
       </c>
+      <c r="R27" s="69" t="n">
+        <v>46050.30069444444</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="67" t="n">
@@ -7829,6 +7916,9 @@
         <f>INT(A28)</f>
         <v/>
       </c>
+      <c r="R28" s="69" t="n">
+        <v>46051.29583333333</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="67" t="n">
@@ -7887,6 +7977,9 @@
         <f>INT(A29)</f>
         <v/>
       </c>
+      <c r="R29" s="69" t="n">
+        <v>46053.44375</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="67" t="n">
@@ -7945,6 +8038,9 @@
         <f>INT(A30)</f>
         <v/>
       </c>
+      <c r="R30" s="69" t="n">
+        <v>46054.44305555556</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="67" t="n">
@@ -8003,6 +8099,9 @@
         <f>INT(A31)</f>
         <v/>
       </c>
+      <c r="R31" s="69" t="n">
+        <v>46055.3125</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="67" t="n">
@@ -8061,6 +8160,9 @@
         <f>INT(A32)</f>
         <v/>
       </c>
+      <c r="R32" s="69" t="n">
+        <v>46056.32430555556</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="67" t="n">
@@ -8119,6 +8221,9 @@
         <f>INT(A33)</f>
         <v/>
       </c>
+      <c r="R33" s="69" t="n">
+        <v>46057.31458333333</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="67" t="n">
@@ -8177,6 +8282,9 @@
         <f>INT(A34)</f>
         <v/>
       </c>
+      <c r="R34" s="69" t="n">
+        <v>46058.325</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="67" t="n">
@@ -8235,6 +8343,9 @@
         <f>INT(A35)</f>
         <v/>
       </c>
+      <c r="R35" s="69" t="n">
+        <v>46059.30763888889</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="67" t="n">
@@ -8293,6 +8404,9 @@
         <f>INT(A36)</f>
         <v/>
       </c>
+      <c r="R36" s="69" t="n">
+        <v>46060.44027777778</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="67" t="n">
@@ -8351,6 +8465,9 @@
         <f>INT(A37)</f>
         <v/>
       </c>
+      <c r="R37" s="69" t="n">
+        <v>46061.45416666667</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="67" t="n">
@@ -8409,6 +8526,9 @@
         <f>INT(A38)</f>
         <v/>
       </c>
+      <c r="R38" s="69" t="n">
+        <v>46062.32708333333</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="67" t="n">
@@ -8467,6 +8587,9 @@
         <f>INT(A39)</f>
         <v/>
       </c>
+      <c r="R39" s="69" t="n">
+        <v>46064.30277777778</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="67" t="n">
@@ -8525,6 +8648,9 @@
         <f>INT(A40)</f>
         <v/>
       </c>
+      <c r="R40" s="69" t="n">
+        <v>46065.32708333333</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="67" t="n">
@@ -8583,6 +8709,9 @@
         <f>INT(A41)</f>
         <v/>
       </c>
+      <c r="R41" s="69" t="n">
+        <v>46066.30138888889</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="67" t="n">
@@ -8641,6 +8770,9 @@
         <f>INT(A42)</f>
         <v/>
       </c>
+      <c r="R42" s="69" t="n">
+        <v>46067.45625</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="67" t="n">
@@ -8699,6 +8831,9 @@
         <f>INT(A43)</f>
         <v/>
       </c>
+      <c r="R43" s="69" t="n">
+        <v>46068.45347222222</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="67" t="n">
@@ -8757,6 +8892,9 @@
         <f>INT(A44)</f>
         <v/>
       </c>
+      <c r="R44" s="69" t="n">
+        <v>46069.325</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="67" t="n">
@@ -8815,6 +8953,9 @@
         <f>INT(A45)</f>
         <v/>
       </c>
+      <c r="R45" s="69" t="n">
+        <v>46070.32361111111</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="67" t="n">
@@ -8873,6 +9014,9 @@
         <f>INT(A46)</f>
         <v/>
       </c>
+      <c r="R46" s="69" t="n">
+        <v>46071.32361111111</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="67" t="n">
@@ -8931,6 +9075,9 @@
         <f>INT(A47)</f>
         <v/>
       </c>
+      <c r="R47" s="69" t="n">
+        <v>46072.32013888889</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="67" t="n">
@@ -8989,6 +9136,9 @@
         <f>INT(A48)</f>
         <v/>
       </c>
+      <c r="R48" s="69" t="n">
+        <v>46073.32083333333</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="67" t="n">
@@ -9047,6 +9197,9 @@
         <f>INT(A49)</f>
         <v/>
       </c>
+      <c r="R49" s="69" t="n">
+        <v>46074.44861111111</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="67" t="n">
@@ -9105,6 +9258,9 @@
         <f>INT(A50)</f>
         <v/>
       </c>
+      <c r="R50" s="69" t="n">
+        <v>46074.45069444444</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="67" t="n">
@@ -9163,6 +9319,9 @@
         <f>INT(A51)</f>
         <v/>
       </c>
+      <c r="R51" s="69" t="n">
+        <v>46075.43541666667</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="67" t="n">
@@ -9221,6 +9380,9 @@
         <f>INT(A52)</f>
         <v/>
       </c>
+      <c r="R52" s="69" t="n">
+        <v>46076.31388888889</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="67" t="n">
@@ -9279,6 +9441,9 @@
         <f>INT(A53)</f>
         <v/>
       </c>
+      <c r="R53" s="69" t="n">
+        <v>46077.30972222222</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="67" t="n">
@@ -9337,6 +9502,9 @@
         <f>INT(A54)</f>
         <v/>
       </c>
+      <c r="R54" s="69" t="n">
+        <v>46078.32777777778</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="67" t="n">
@@ -9395,6 +9563,9 @@
         <f>INT(A55)</f>
         <v/>
       </c>
+      <c r="R55" s="69" t="n">
+        <v>46079.31388888889</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="67" t="n">
@@ -9453,6 +9624,9 @@
         <f>INT(A56)</f>
         <v/>
       </c>
+      <c r="R56" s="69" t="n">
+        <v>46080.31805555556</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="67" t="n">
@@ -9511,6 +9685,9 @@
         <f>INT(A57)</f>
         <v/>
       </c>
+      <c r="R57" s="69" t="n">
+        <v>46081.4375</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="67" t="n">
@@ -9569,6 +9746,9 @@
         <f>INT(A58)</f>
         <v/>
       </c>
+      <c r="R58" s="69" t="n">
+        <v>46082.4375</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="67" t="n">
@@ -9627,6 +9807,9 @@
         <f>INT(A59)</f>
         <v/>
       </c>
+      <c r="R59" s="69" t="n">
+        <v>46083.30208333334</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="67" t="n">
@@ -9685,6 +9868,9 @@
         <f>INT(A60)</f>
         <v/>
       </c>
+      <c r="R60" s="69" t="n">
+        <v>46085.29444444444</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="67" t="n">
@@ -9743,6 +9929,9 @@
         <f>INT(A61)</f>
         <v/>
       </c>
+      <c r="R61" s="69" t="n">
+        <v>46086.31388888889</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="67" t="n">
@@ -9801,6 +9990,9 @@
         <f>INT(A62)</f>
         <v/>
       </c>
+      <c r="R62" s="69" t="n">
+        <v>46087.30208333334</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="67" t="n">
@@ -9859,6 +10051,9 @@
         <f>INT(A63)</f>
         <v/>
       </c>
+      <c r="R63" s="69" t="n">
+        <v>46088.42777777778</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="67" t="n">
@@ -9917,6 +10112,9 @@
         <f>INT(A64)</f>
         <v/>
       </c>
+      <c r="R64" s="69" t="n">
+        <v>46089.43402777778</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="67" t="n">
@@ -9975,6 +10173,9 @@
         <f>INT(A65)</f>
         <v/>
       </c>
+      <c r="R65" s="69" t="n">
+        <v>46090.29444444444</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="67" t="n">
@@ -10033,6 +10234,9 @@
         <f>INT(A66)</f>
         <v/>
       </c>
+      <c r="R66" s="69" t="n">
+        <v>46091.32013888889</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="67" t="n">
@@ -10091,6 +10295,9 @@
         <f>INT(A67)</f>
         <v/>
       </c>
+      <c r="R67" s="69" t="n">
+        <v>46092.31180555555</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="67" t="n">
@@ -10149,6 +10356,9 @@
         <f>INT(A68)</f>
         <v/>
       </c>
+      <c r="R68" s="69" t="n">
+        <v>46093.32847222222</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="67" t="n">
@@ -10207,6 +10417,9 @@
         <f>INT(A69)</f>
         <v/>
       </c>
+      <c r="R69" s="69" t="n">
+        <v>46094.30902777778</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="67" t="n">
@@ -10265,6 +10478,9 @@
         <f>INT(A70)</f>
         <v/>
       </c>
+      <c r="R70" s="69" t="n">
+        <v>46096.43611111111</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="67" t="n">
@@ -10323,6 +10539,9 @@
         <f>INT(A71)</f>
         <v/>
       </c>
+      <c r="R71" s="69" t="n">
+        <v>46097.30416666667</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="67" t="n">
@@ -10381,6 +10600,9 @@
         <f>INT(A72)</f>
         <v/>
       </c>
+      <c r="R72" s="69" t="n">
+        <v>46098.29583333333</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="67" t="n">
@@ -10439,6 +10661,9 @@
         <f>INT(A73)</f>
         <v/>
       </c>
+      <c r="R73" s="69" t="n">
+        <v>46099.29930555556</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="67" t="n">
@@ -10497,6 +10722,9 @@
         <f>INT(A74)</f>
         <v/>
       </c>
+      <c r="R74" s="69" t="n">
+        <v>46100.30277777778</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="67" t="n">
@@ -10555,6 +10783,9 @@
         <f>INT(A75)</f>
         <v/>
       </c>
+      <c r="R75" s="69" t="n">
+        <v>46101.31319444445</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="67" t="n">
@@ -10613,6 +10844,9 @@
         <f>INT(A76)</f>
         <v/>
       </c>
+      <c r="R76" s="69" t="n">
+        <v>46102.41944444444</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="67" t="n">
@@ -10671,6 +10905,9 @@
         <f>INT(A77)</f>
         <v/>
       </c>
+      <c r="R77" s="69" t="n">
+        <v>46103.42777777778</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="67" t="n">
@@ -10729,6 +10966,9 @@
         <f>INT(A78)</f>
         <v/>
       </c>
+      <c r="R78" s="69" t="n">
+        <v>46104.30625</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="67" t="n">
@@ -10787,6 +11027,9 @@
         <f>INT(A79)</f>
         <v/>
       </c>
+      <c r="R79" s="69" t="n">
+        <v>46105.31875</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="67" t="n">
@@ -10845,6 +11088,9 @@
         <f>INT(A80)</f>
         <v/>
       </c>
+      <c r="R80" s="69" t="n">
+        <v>46105.32083333333</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="67" t="n">
@@ -10903,6 +11149,9 @@
         <f>INT(A81)</f>
         <v/>
       </c>
+      <c r="R81" s="69" t="n">
+        <v>46106.29375</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="67" t="n">
@@ -10961,6 +11210,9 @@
         <f>INT(A82)</f>
         <v/>
       </c>
+      <c r="R82" s="69" t="n">
+        <v>46107.31458333333</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="67" t="n">
@@ -11019,6 +11271,9 @@
         <f>INT(A83)</f>
         <v/>
       </c>
+      <c r="R83" s="69" t="n">
+        <v>46108.29236111111</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="67" t="n">
@@ -11077,6 +11332,9 @@
         <f>INT(A84)</f>
         <v/>
       </c>
+      <c r="R84" s="69" t="n">
+        <v>46110.38333333333</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="67" t="n">
@@ -11135,6 +11393,9 @@
         <f>INT(A85)</f>
         <v/>
       </c>
+      <c r="R85" s="69" t="n">
+        <v>46111.27916666667</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="67" t="n">
@@ -11193,6 +11454,9 @@
         <f>INT(A86)</f>
         <v/>
       </c>
+      <c r="R86" s="69" t="n">
+        <v>46112.27222222222</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="67" t="n">
@@ -11251,6 +11515,9 @@
         <f>INT(A87)</f>
         <v/>
       </c>
+      <c r="R87" s="69" t="n">
+        <v>46113.28194444445</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="67" t="n">
@@ -11309,6 +11576,9 @@
         <f>INT(A88)</f>
         <v/>
       </c>
+      <c r="R88" s="69" t="n">
+        <v>46114.25208333333</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="67" t="n">
@@ -11367,6 +11637,9 @@
         <f>INT(A89)</f>
         <v/>
       </c>
+      <c r="R89" s="69" t="n">
+        <v>46115.25208333333</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="67" t="n">
@@ -11425,6 +11698,9 @@
         <f>INT(A90)</f>
         <v/>
       </c>
+      <c r="R90" s="69" t="n">
+        <v>46116.40416666667</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="67" t="n">
@@ -11483,6 +11759,9 @@
         <f>INT(A91)</f>
         <v/>
       </c>
+      <c r="R91" s="69" t="n">
+        <v>46117.38680555556</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="67" t="n">
@@ -11541,6 +11820,9 @@
         <f>INT(A92)</f>
         <v/>
       </c>
+      <c r="R92" s="69" t="n">
+        <v>46118.27430555555</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="67" t="n">
@@ -11599,6 +11881,9 @@
         <f>INT(A93)</f>
         <v/>
       </c>
+      <c r="R93" s="69" t="n">
+        <v>46119.26458333333</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="67" t="n">
@@ -11657,6 +11942,9 @@
         <f>INT(A94)</f>
         <v/>
       </c>
+      <c r="R94" s="69" t="n">
+        <v>46120.25833333333</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="67" t="n">
@@ -11715,6 +12003,9 @@
         <f>INT(A95)</f>
         <v/>
       </c>
+      <c r="R95" s="69" t="n">
+        <v>46121.27569444444</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="67" t="n">
@@ -11773,6 +12064,9 @@
         <f>INT(A96)</f>
         <v/>
       </c>
+      <c r="R96" s="69" t="n">
+        <v>46122.25972222222</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="67" t="n">
@@ -11831,6 +12125,9 @@
         <f>INT(A97)</f>
         <v/>
       </c>
+      <c r="R97" s="69" t="n">
+        <v>46123.40972222222</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="67" t="n">
@@ -11889,6 +12186,9 @@
         <f>INT(A98)</f>
         <v/>
       </c>
+      <c r="R98" s="69" t="n">
+        <v>46124.39652777778</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="67" t="n">
@@ -11947,6 +12247,9 @@
         <f>INT(A99)</f>
         <v/>
       </c>
+      <c r="R99" s="69" t="n">
+        <v>46125.28958333333</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="67" t="n">
@@ -12005,6 +12308,9 @@
         <f>INT(A100)</f>
         <v/>
       </c>
+      <c r="R100" s="69" t="n">
+        <v>46126.27222222222</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="67" t="n">
@@ -12063,6 +12369,9 @@
         <f>INT(A101)</f>
         <v/>
       </c>
+      <c r="R101" s="69" t="n">
+        <v>46127.28611111111</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="67" t="n">
@@ -12121,6 +12430,9 @@
         <f>INT(A102)</f>
         <v/>
       </c>
+      <c r="R102" s="69" t="n">
+        <v>46128.28055555555</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="67" t="n">
@@ -12179,6 +12491,9 @@
         <f>INT(A103)</f>
         <v/>
       </c>
+      <c r="R103" s="69" t="n">
+        <v>46129.26666666667</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="67" t="n">
@@ -12237,6 +12552,9 @@
         <f>INT(A104)</f>
         <v/>
       </c>
+      <c r="R104" s="69" t="n">
+        <v>46130.40277777778</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="67" t="n">
@@ -12295,6 +12613,9 @@
         <f>INT(A105)</f>
         <v/>
       </c>
+      <c r="R105" s="69" t="n">
+        <v>46132.28958333333</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="67" t="n">
@@ -12353,6 +12674,9 @@
         <f>INT(A106)</f>
         <v/>
       </c>
+      <c r="R106" s="69" t="n">
+        <v>46134.26111111111</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="67" t="n">
@@ -12411,6 +12735,9 @@
         <f>INT(A107)</f>
         <v/>
       </c>
+      <c r="R107" s="69" t="n">
+        <v>46135.27847222222</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="67" t="n">
@@ -12469,6 +12796,9 @@
         <f>INT(A108)</f>
         <v/>
       </c>
+      <c r="R108" s="69" t="n">
+        <v>46136.27083333334</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="67" t="n">
@@ -12527,6 +12857,9 @@
         <f>INT(A109)</f>
         <v/>
       </c>
+      <c r="R109" s="69" t="n">
+        <v>46136.27291666667</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="67" t="n">
@@ -12585,6 +12918,9 @@
         <f>INT(A110)</f>
         <v/>
       </c>
+      <c r="R110" s="69" t="n">
+        <v>46137.40138888889</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="67" t="n">
@@ -12643,6 +12979,9 @@
         <f>INT(A111)</f>
         <v/>
       </c>
+      <c r="R111" s="69" t="n">
+        <v>46138.38819444444</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="67" t="n">
@@ -12701,6 +13040,9 @@
         <f>INT(A112)</f>
         <v/>
       </c>
+      <c r="R112" s="69" t="n">
+        <v>46139.25416666667</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="67" t="n">
@@ -12759,6 +13101,9 @@
         <f>INT(A113)</f>
         <v/>
       </c>
+      <c r="R113" s="69" t="n">
+        <v>46140.27291666667</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="67" t="n">
@@ -12817,6 +13162,9 @@
         <f>INT(A114)</f>
         <v/>
       </c>
+      <c r="R114" s="69" t="n">
+        <v>46141.26319444444</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="67" t="n">
@@ -12875,6 +13223,9 @@
         <f>INT(A115)</f>
         <v/>
       </c>
+      <c r="R115" s="69" t="n">
+        <v>46143.28611111111</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="67" t="n">
@@ -12933,6 +13284,9 @@
         <f>INT(A116)</f>
         <v/>
       </c>
+      <c r="R116" s="69" t="n">
+        <v>46144.41597222222</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="67" t="n">
@@ -12991,6 +13345,9 @@
         <f>INT(A117)</f>
         <v/>
       </c>
+      <c r="R117" s="69" t="n">
+        <v>46145.39791666667</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="67" t="n">
@@ -13049,6 +13406,9 @@
         <f>INT(A118)</f>
         <v/>
       </c>
+      <c r="R118" s="69" t="n">
+        <v>46146.25486111111</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="67" t="n">
@@ -13107,6 +13467,9 @@
         <f>INT(A119)</f>
         <v/>
       </c>
+      <c r="R119" s="69" t="n">
+        <v>46147.27152777778</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="67" t="n">
@@ -13165,6 +13528,9 @@
         <f>INT(A120)</f>
         <v/>
       </c>
+      <c r="R120" s="69" t="n">
+        <v>46148.28194444445</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="67" t="n">
@@ -13223,6 +13589,9 @@
         <f>INT(A121)</f>
         <v/>
       </c>
+      <c r="R121" s="69" t="n">
+        <v>46149.28680555556</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="67" t="n">
@@ -13281,6 +13650,9 @@
         <f>INT(A122)</f>
         <v/>
       </c>
+      <c r="R122" s="69" t="n">
+        <v>46150.25833333333</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="67" t="n">
@@ -13339,6 +13711,9 @@
         <f>INT(A123)</f>
         <v/>
       </c>
+      <c r="R123" s="69" t="n">
+        <v>46151.39097222222</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="67" t="n">
@@ -13397,6 +13772,9 @@
         <f>INT(A124)</f>
         <v/>
       </c>
+      <c r="R124" s="69" t="n">
+        <v>46152.40833333333</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="67" t="n">
@@ -13455,6 +13833,9 @@
         <f>INT(A125)</f>
         <v/>
       </c>
+      <c r="R125" s="69" t="n">
+        <v>46153.28680555556</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="67" t="n">
@@ -13513,6 +13894,9 @@
         <f>INT(A126)</f>
         <v/>
       </c>
+      <c r="R126" s="69" t="n">
+        <v>46154.26388888889</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="67" t="n">
@@ -13571,6 +13955,9 @@
         <f>INT(A127)</f>
         <v/>
       </c>
+      <c r="R127" s="69" t="n">
+        <v>46155.28888888889</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="67" t="n">
@@ -13629,6 +14016,9 @@
         <f>INT(A128)</f>
         <v/>
       </c>
+      <c r="R128" s="69" t="n">
+        <v>46156.25902777778</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="67" t="n">
@@ -13687,6 +14077,9 @@
         <f>INT(A129)</f>
         <v/>
       </c>
+      <c r="R129" s="69" t="n">
+        <v>46157.26944444444</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="67" t="n">
@@ -13745,6 +14138,9 @@
         <f>INT(A130)</f>
         <v/>
       </c>
+      <c r="R130" s="69" t="n">
+        <v>46158.39930555555</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="67" t="n">
@@ -13803,6 +14199,9 @@
         <f>INT(A131)</f>
         <v/>
       </c>
+      <c r="R131" s="69" t="n">
+        <v>46159.38819444444</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="67" t="n">
@@ -13861,6 +14260,9 @@
         <f>INT(A132)</f>
         <v/>
       </c>
+      <c r="R132" s="69" t="n">
+        <v>46160.27083333334</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="67" t="n">
@@ -13919,6 +14321,9 @@
         <f>INT(A133)</f>
         <v/>
       </c>
+      <c r="R133" s="69" t="n">
+        <v>46161.25694444445</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="67" t="n">
@@ -13977,6 +14382,9 @@
         <f>INT(A134)</f>
         <v/>
       </c>
+      <c r="R134" s="69" t="n">
+        <v>46162.26458333333</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="67" t="n">
@@ -14035,6 +14443,9 @@
         <f>INT(A135)</f>
         <v/>
       </c>
+      <c r="R135" s="69" t="n">
+        <v>46163.25833333333</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="67" t="n">
@@ -14093,6 +14504,9 @@
         <f>INT(A136)</f>
         <v/>
       </c>
+      <c r="R136" s="69" t="n">
+        <v>46164.28541666667</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="67" t="n">
@@ -14151,6 +14565,9 @@
         <f>INT(A137)</f>
         <v/>
       </c>
+      <c r="R137" s="69" t="n">
+        <v>46165.39305555556</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="67" t="n">
@@ -14209,6 +14626,9 @@
         <f>INT(A138)</f>
         <v/>
       </c>
+      <c r="R138" s="69" t="n">
+        <v>46166.39652777778</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="67" t="n">
@@ -14267,6 +14687,9 @@
         <f>INT(A139)</f>
         <v/>
       </c>
+      <c r="R139" s="69" t="n">
+        <v>46167.27222222222</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="67" t="n">
@@ -14325,6 +14748,9 @@
         <f>INT(A140)</f>
         <v/>
       </c>
+      <c r="R140" s="69" t="n">
+        <v>46167.27430555555</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="67" t="n">
@@ -14383,6 +14809,9 @@
         <f>INT(A141)</f>
         <v/>
       </c>
+      <c r="R141" s="69" t="n">
+        <v>46168.26666666667</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="67" t="n">
@@ -14441,6 +14870,9 @@
         <f>INT(A142)</f>
         <v/>
       </c>
+      <c r="R142" s="69" t="n">
+        <v>46169.2875</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="67" t="n">
@@ -14499,6 +14931,9 @@
         <f>INT(A143)</f>
         <v/>
       </c>
+      <c r="R143" s="69" t="n">
+        <v>46170.28541666667</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="67" t="n">
@@ -14557,6 +14992,9 @@
         <f>INT(A144)</f>
         <v/>
       </c>
+      <c r="R144" s="69" t="n">
+        <v>46172.41597222222</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="67" t="n">
@@ -14615,6 +15053,9 @@
         <f>INT(A145)</f>
         <v/>
       </c>
+      <c r="R145" s="69" t="n">
+        <v>46173.38472222222</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="67" t="n">
@@ -14673,6 +15114,9 @@
         <f>INT(A146)</f>
         <v/>
       </c>
+      <c r="R146" s="69" t="n">
+        <v>46174.28611111111</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="67" t="n">
@@ -14731,11 +15175,14 @@
         <f>INT(A147)</f>
         <v/>
       </c>
+      <c r="R147" s="69" t="n">
+        <v>46175.25138888889</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
@@ -14774,7 +15221,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:46</t>
+          <t>Atualizado em 11/10/2026 12:56</t>
         </is>
       </c>
     </row>
@@ -14811,774 +15258,774 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="69" t="inlineStr">
+      <c r="A4" s="70" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="B4" s="69" t="inlineStr">
+      <c r="B4" s="70" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C4" s="69" t="inlineStr">
+      <c r="C4" s="70" t="inlineStr">
         <is>
           <t>Peso medido pela balança</t>
         </is>
       </c>
-      <c r="D4" s="69" t="inlineStr">
+      <c r="D4" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E4" s="69" t="inlineStr">
+      <c r="E4" s="70" t="inlineStr">
         <is>
           <t>balança</t>
         </is>
       </c>
-      <c r="F4" s="69" t="inlineStr">
+      <c r="F4" s="70" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="69" t="inlineStr">
+      <c r="A5" s="70" t="inlineStr">
         <is>
           <t>Altura</t>
         </is>
       </c>
-      <c r="B5" s="69" t="inlineStr">
+      <c r="B5" s="70" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="C5" s="69" t="inlineStr">
+      <c r="C5" s="70" t="inlineStr">
         <is>
           <t>Altura do perfil associada à leitura</t>
         </is>
       </c>
-      <c r="D5" s="69" t="inlineStr">
+      <c r="D5" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E5" s="69" t="inlineStr">
+      <c r="E5" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F5" s="69" t="inlineStr">
+      <c r="F5" s="70" t="inlineStr">
         <is>
           <t>Height</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="69" t="inlineStr">
+      <c r="A6" s="70" t="inlineStr">
         <is>
           <t>IMC</t>
         </is>
       </c>
-      <c r="B6" s="69" t="inlineStr">
+      <c r="B6" s="70" t="inlineStr">
         <is>
           <t>kg/m²</t>
         </is>
       </c>
-      <c r="C6" s="69" t="inlineStr">
+      <c r="C6" s="70" t="inlineStr">
         <is>
           <t>Índice de massa corporal</t>
         </is>
       </c>
-      <c r="D6" s="69" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E6" s="69" t="inlineStr">
+      <c r="E6" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F6" s="69" t="inlineStr">
+      <c r="F6" s="70" t="inlineStr">
         <is>
           <t>BMI</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="69" t="inlineStr">
+      <c r="A7" s="70" t="inlineStr">
         <is>
           <t>Gordura corporal</t>
         </is>
       </c>
-      <c r="B7" s="69" t="inlineStr">
+      <c r="B7" s="70" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C7" s="69" t="inlineStr">
+      <c r="C7" s="70" t="inlineStr">
         <is>
           <t>Estimativa por bioimpedância</t>
         </is>
       </c>
-      <c r="D7" s="69" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E7" s="69" t="inlineStr">
+      <c r="E7" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F7" s="69" t="inlineStr">
+      <c r="F7" s="70" t="inlineStr">
         <is>
           <t>BodyFat</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="69" t="inlineStr">
+      <c r="A8" s="70" t="inlineStr">
         <is>
           <t>Água corporal</t>
         </is>
       </c>
-      <c r="B8" s="69" t="inlineStr">
+      <c r="B8" s="70" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C8" s="69" t="inlineStr">
+      <c r="C8" s="70" t="inlineStr">
         <is>
           <t>Estimativa de água corporal</t>
         </is>
       </c>
-      <c r="D8" s="69" t="inlineStr">
+      <c r="D8" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E8" s="69" t="inlineStr">
+      <c r="E8" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F8" s="69" t="inlineStr">
+      <c r="F8" s="70" t="inlineStr">
         <is>
           <t>BodyWater</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="69" t="inlineStr">
+      <c r="A9" s="70" t="inlineStr">
         <is>
           <t>Massa óssea</t>
         </is>
       </c>
-      <c r="B9" s="69" t="inlineStr">
+      <c r="B9" s="70" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C9" s="69" t="inlineStr">
+      <c r="C9" s="70" t="inlineStr">
         <is>
           <t>Estimativa; não é densidade mineral óssea</t>
         </is>
       </c>
-      <c r="D9" s="69" t="inlineStr">
+      <c r="D9" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E9" s="69" t="inlineStr">
+      <c r="E9" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F9" s="69" t="inlineStr">
+      <c r="F9" s="70" t="inlineStr">
         <is>
           <t>BoneMass</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="69" t="inlineStr">
+      <c r="A10" s="70" t="inlineStr">
         <is>
           <t>Massa muscular</t>
         </is>
       </c>
-      <c r="B10" s="69" t="inlineStr">
+      <c r="B10" s="70" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C10" s="69" t="inlineStr">
+      <c r="C10" s="70" t="inlineStr">
         <is>
           <t>Estimativa de massa muscular</t>
         </is>
       </c>
-      <c r="D10" s="69" t="inlineStr">
+      <c r="D10" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E10" s="69" t="inlineStr">
+      <c r="E10" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F10" s="69" t="inlineStr">
+      <c r="F10" s="70" t="inlineStr">
         <is>
           <t>MuscleMass</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="69" t="inlineStr">
+      <c r="A11" s="70" t="inlineStr">
         <is>
           <t>Proteína</t>
         </is>
       </c>
-      <c r="B11" s="69" t="inlineStr">
+      <c r="B11" s="70" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C11" s="69" t="inlineStr">
+      <c r="C11" s="70" t="inlineStr">
         <is>
           <t>Proporção estimada de proteína</t>
         </is>
       </c>
-      <c r="D11" s="69" t="inlineStr">
+      <c r="D11" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E11" s="69" t="inlineStr">
+      <c r="E11" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F11" s="69" t="inlineStr">
+      <c r="F11" s="70" t="inlineStr">
         <is>
           <t>ProteinRatio</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="69" t="inlineStr">
+      <c r="A12" s="70" t="inlineStr">
         <is>
           <t>Massa proteica</t>
         </is>
       </c>
-      <c r="B12" s="69" t="inlineStr">
+      <c r="B12" s="70" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C12" s="69" t="inlineStr">
+      <c r="C12" s="70" t="inlineStr">
         <is>
           <t>Derivada pelo leitor: peso × proteína / 100</t>
         </is>
       </c>
-      <c r="D12" s="69" t="inlineStr">
+      <c r="D12" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E12" s="69" t="inlineStr">
+      <c r="E12" s="70" t="inlineStr">
         <is>
           <t>derivada</t>
         </is>
       </c>
-      <c r="F12" s="69" t="inlineStr">
+      <c r="F12" s="70" t="inlineStr">
         <is>
           <t>ProteinMass</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="69" t="inlineStr">
+      <c r="A13" s="70" t="inlineStr">
         <is>
           <t>Gordura visceral</t>
         </is>
       </c>
-      <c r="B13" s="69" t="inlineStr">
+      <c r="B13" s="70" t="inlineStr">
         <is>
           <t>índice</t>
         </is>
       </c>
-      <c r="C13" s="69" t="inlineStr">
+      <c r="C13" s="70" t="inlineStr">
         <is>
           <t>Índice da aplicação; não é percentagem (inteiro no leitor)</t>
         </is>
       </c>
-      <c r="D13" s="69" t="inlineStr">
+      <c r="D13" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E13" s="69" t="inlineStr">
+      <c r="E13" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F13" s="69" t="inlineStr">
+      <c r="F13" s="70" t="inlineStr">
         <is>
           <t>VisceralFat</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="69" t="inlineStr">
+      <c r="A14" s="70" t="inlineStr">
         <is>
           <t>Metabolismo basal</t>
         </is>
       </c>
-      <c r="B14" s="69" t="inlineStr">
+      <c r="B14" s="70" t="inlineStr">
         <is>
           <t>kcal/dia</t>
         </is>
       </c>
-      <c r="C14" s="69" t="inlineStr">
+      <c r="C14" s="70" t="inlineStr">
         <is>
           <t>Estimativa de gasto basal (inteiro no leitor)</t>
         </is>
       </c>
-      <c r="D14" s="69" t="inlineStr">
+      <c r="D14" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E14" s="69" t="inlineStr">
+      <c r="E14" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F14" s="69" t="inlineStr">
+      <c r="F14" s="70" t="inlineStr">
         <is>
           <t>BasalMetabolism</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="69" t="inlineStr">
+      <c r="A15" s="70" t="inlineStr">
         <is>
           <t>Idade corporal</t>
         </is>
       </c>
-      <c r="B15" s="69" t="inlineStr">
+      <c r="B15" s="70" t="inlineStr">
         <is>
           <t>anos</t>
         </is>
       </c>
-      <c r="C15" s="69" t="inlineStr">
+      <c r="C15" s="70" t="inlineStr">
         <is>
           <t>Estimativa; não é idade cronológica</t>
         </is>
       </c>
-      <c r="D15" s="69" t="inlineStr">
+      <c r="D15" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E15" s="69" t="inlineStr">
+      <c r="E15" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F15" s="69" t="inlineStr">
+      <c r="F15" s="70" t="inlineStr">
         <is>
           <t>MetabolicAge</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="69" t="inlineStr">
+      <c r="A16" s="70" t="inlineStr">
         <is>
           <t>Pontuação corporal</t>
         </is>
       </c>
-      <c r="B16" s="69" t="inlineStr">
+      <c r="B16" s="70" t="inlineStr">
         <is>
           <t>pontos</t>
         </is>
       </c>
-      <c r="C16" s="69" t="inlineStr">
+      <c r="C16" s="70" t="inlineStr">
         <is>
           <t>Pontuação global da aplicação</t>
         </is>
       </c>
-      <c r="D16" s="69" t="inlineStr">
+      <c r="D16" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E16" s="69" t="inlineStr">
+      <c r="E16" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F16" s="69" t="inlineStr">
+      <c r="F16" s="70" t="inlineStr">
         <is>
           <t>BodyScore</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="69" t="inlineStr">
+      <c r="A17" s="70" t="inlineStr">
         <is>
           <t>Classificação física</t>
         </is>
       </c>
-      <c r="B17" s="69" t="inlineStr">
+      <c r="B17" s="70" t="inlineStr">
         <is>
           <t>código</t>
         </is>
       </c>
-      <c r="C17" s="69" t="inlineStr">
+      <c r="C17" s="70" t="inlineStr">
         <is>
           <t>Código original, sem interpretação documentada</t>
         </is>
       </c>
-      <c r="D17" s="69" t="inlineStr">
+      <c r="D17" s="70" t="inlineStr">
         <is>
           <t>0 de 144 leituras</t>
         </is>
       </c>
-      <c r="E17" s="69" t="inlineStr">
+      <c r="E17" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F17" s="69" t="inlineStr">
+      <c r="F17" s="70" t="inlineStr">
         <is>
           <t>PhysiqueRating</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="69" t="inlineStr">
+      <c r="A18" s="70" t="inlineStr">
         <is>
           <t>Peso padrão</t>
         </is>
       </c>
-      <c r="B18" s="69" t="inlineStr">
+      <c r="B18" s="70" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C18" s="69" t="inlineStr">
+      <c r="C18" s="70" t="inlineStr">
         <is>
           <t>Referência da aplicação; não é um objetivo individual</t>
         </is>
       </c>
-      <c r="D18" s="69" t="inlineStr">
+      <c r="D18" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E18" s="69" t="inlineStr">
+      <c r="E18" s="70" t="inlineStr">
         <is>
           <t>aplicação</t>
         </is>
       </c>
-      <c r="F18" s="69" t="inlineStr">
+      <c r="F18" s="70" t="inlineStr">
         <is>
           <t>StandBodyWeight</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="69" t="inlineStr">
+      <c r="A19" s="70" t="inlineStr">
         <is>
           <t>Impedância</t>
         </is>
       </c>
-      <c r="B19" s="69" t="inlineStr">
+      <c r="B19" s="70" t="inlineStr">
         <is>
           <t>Ω</t>
         </is>
       </c>
-      <c r="C19" s="69" t="inlineStr">
+      <c r="C19" s="70" t="inlineStr">
         <is>
           <t>Impedância registada pela balança</t>
         </is>
       </c>
-      <c r="D19" s="69" t="inlineStr">
+      <c r="D19" s="70" t="inlineStr">
         <is>
           <t>144 de 144 leituras</t>
         </is>
       </c>
-      <c r="E19" s="69" t="inlineStr">
+      <c r="E19" s="70" t="inlineStr">
         <is>
           <t>balança</t>
         </is>
       </c>
-      <c r="F19" s="69" t="inlineStr">
+      <c r="F19" s="70" t="inlineStr">
         <is>
           <t>Impedance</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="69" t="inlineStr">
+      <c r="A20" s="70" t="inlineStr">
         <is>
           <t>Massa gorda</t>
         </is>
       </c>
-      <c r="B20" s="69" t="inlineStr">
+      <c r="B20" s="70" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C20" s="69" t="inlineStr">
+      <c r="C20" s="70" t="inlineStr">
         <is>
           <t>Peso × gordura / 100</t>
         </is>
       </c>
-      <c r="D20" s="69" t="inlineStr">
+      <c r="D20" s="70" t="inlineStr">
         <is>
           <t>144 leituras</t>
         </is>
       </c>
-      <c r="E20" s="69" t="inlineStr">
+      <c r="E20" s="70" t="inlineStr">
         <is>
           <t>derivada</t>
         </is>
       </c>
-      <c r="F20" s="69" t="inlineStr">
+      <c r="F20" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="69" t="inlineStr">
+      <c r="A21" s="70" t="inlineStr">
         <is>
           <t>Médias de 7 dias</t>
         </is>
       </c>
-      <c r="B21" s="69" t="inlineStr">
+      <c r="B21" s="70" t="inlineStr">
         <is>
           <t>kg / %</t>
         </is>
       </c>
-      <c r="C21" s="69" t="inlineStr">
+      <c r="C21" s="70" t="inlineStr">
         <is>
           <t>Média das leituras em ]t − 7 dias, t]</t>
         </is>
       </c>
-      <c r="D21" s="69" t="inlineStr">
+      <c r="D21" s="70" t="inlineStr">
         <is>
           <t>144 leituras</t>
         </is>
       </c>
-      <c r="E21" s="69" t="inlineStr">
+      <c r="E21" s="70" t="inlineStr">
         <is>
           <t>derivada</t>
         </is>
       </c>
-      <c r="F21" s="69" t="inlineStr">
+      <c r="F21" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="69" t="inlineStr">
+      <c r="A22" s="70" t="inlineStr">
         <is>
           <t>Cintura</t>
         </is>
       </c>
-      <c r="B22" s="69" t="inlineStr">
+      <c r="B22" s="70" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="C22" s="69" t="inlineStr">
+      <c r="C22" s="70" t="inlineStr">
         <is>
           <t>Circunferência ao nível do umbigo (média de 3 leituras)</t>
         </is>
       </c>
-      <c r="D22" s="69" t="inlineStr">
+      <c r="D22" s="70" t="inlineStr">
         <is>
           <t>17 de 22 semanas</t>
         </is>
       </c>
-      <c r="E22" s="69" t="inlineStr">
+      <c r="E22" s="70" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="F22" s="69" t="inlineStr">
+      <c r="F22" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="69" t="inlineStr">
+      <c r="A23" s="70" t="inlineStr">
         <is>
           <t>Pescoço</t>
         </is>
       </c>
-      <c r="B23" s="69" t="inlineStr">
+      <c r="B23" s="70" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="C23" s="69" t="inlineStr">
+      <c r="C23" s="70" t="inlineStr">
         <is>
           <t>Circunferência do pescoço (média de 3 leituras)</t>
         </is>
       </c>
-      <c r="D23" s="69" t="inlineStr">
+      <c r="D23" s="70" t="inlineStr">
         <is>
           <t>17 de 22 semanas</t>
         </is>
       </c>
-      <c r="E23" s="69" t="inlineStr">
+      <c r="E23" s="70" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="F23" s="69" t="inlineStr">
+      <c r="F23" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="70" t="inlineStr">
+      <c r="A25" s="71" t="inlineStr">
         <is>
           <t>Regras</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="71" t="inlineStr">
+      <c r="A26" s="72" t="inlineStr">
         <is>
           <t>Início</t>
         </is>
       </c>
-      <c r="B26" s="72" t="inlineStr">
+      <c r="B26" s="73" t="inlineStr">
         <is>
           <t>Leituras com data local a partir de 04/01/2026 (Europe/Lisbon).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="71" t="inlineStr">
+      <c r="A27" s="72" t="inlineStr">
         <is>
           <t>Protocolo de pesagem</t>
         </is>
       </c>
-      <c r="B27" s="72" t="inlineStr">
+      <c r="B27" s="73" t="inlineStr">
         <is>
           <t>Ao acordar, depois de ir à casa de banho.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="71" t="inlineStr">
+      <c r="A28" s="72" t="inlineStr">
         <is>
           <t>Perfil</t>
         </is>
       </c>
-      <c r="B28" s="72" t="inlineStr">
+      <c r="B28" s="73" t="inlineStr">
         <is>
           <t>Titular: identificador Zepp -1 (o leitor pede apenas este membro). Exportações antigas sem identificador: altura 178 cm.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="71" t="inlineStr">
+      <c r="A29" s="72" t="inlineStr">
         <is>
           <t>Composição completa</t>
         </is>
       </c>
-      <c r="B29" s="72" t="inlineStr">
+      <c r="B29" s="73" t="inlineStr">
         <is>
           <t>IMC, gordura, água, massa óssea, metabolismo, músculo, visceral, proteína, massa proteica, idade corporal e pontuação com valores numéricos.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="71" t="inlineStr">
+      <c r="A30" s="72" t="inlineStr">
         <is>
           <t>Plausibilidade</t>
         </is>
       </c>
-      <c r="B30" s="72" t="inlineStr">
+      <c r="B30" s="73" t="inlineStr">
         <is>
           <t>Weight 30–250; BMI 10–60; BodyFat 2–70; BodyWater 25–80; BoneMass 0.5–8; MuscleMass 15–150; ProteinRatio 5–35; VisceralFat 1–59; BasalMetabolism 700–4500; MetabolicAge 10–100; BodyScore 0–100</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="71" t="inlineStr">
+      <c r="A31" s="72" t="inlineStr">
         <is>
           <t>Semanas</t>
         </is>
       </c>
-      <c r="B31" s="72" t="inlineStr">
+      <c r="B31" s="73" t="inlineStr">
         <is>
           <t>Domingo a sábado, em hora local.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="71" t="inlineStr">
+      <c r="A32" s="72" t="inlineStr">
         <is>
           <t>Médias</t>
         </is>
       </c>
-      <c r="B32" s="72" t="inlineStr">
+      <c r="B32" s="73" t="inlineStr">
         <is>
           <t>Por leitura (não por dia). 'Dias com medição' mostra quantos dias distintos contribuíram.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="71" t="inlineStr">
+      <c r="A33" s="72" t="inlineStr">
         <is>
           <t>Contagens</t>
         </is>
       </c>
-      <c r="B33" s="72" t="inlineStr">
+      <c r="B33" s="73" t="inlineStr">
         <is>
           <t>origem 155 · anteriores ao início 5 · incompletas 6 · implausíveis 0 · outro perfil 0 · aceites 144</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="71" t="inlineStr">
+      <c r="A34" s="72" t="inlineStr">
         <is>
           <t>Limites</t>
         </is>
       </c>
-      <c r="B34" s="72" t="inlineStr">
+      <c r="B34" s="73" t="inlineStr">
         <is>
           <t>Composição, idade e pontuação são estimativas da aplicação, não diagnósticos clínicos.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="71" t="inlineStr">
+      <c r="A35" s="72" t="inlineStr">
         <is>
           <t>Atualização</t>
         </is>
       </c>
-      <c r="B35" s="72" t="inlineStr">
+      <c r="B35" s="73" t="inlineStr">
         <is>
           <t>Sincronizar a Zepp Life, guardar e fechar o Excel e executar ATUALIZAR-EXCEL.cmd. Depois de editar só medidas manuais: RECALCULAR-SEM-DESCARREGAR.cmd.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="70" t="inlineStr">
+      <c r="A37" s="71" t="inlineStr">
         <is>
           <t>Pesagens excluídas desde o início (6)</t>
         </is>
@@ -15602,78 +16049,78 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="73" t="n">
+      <c r="A39" s="74" t="n">
         <v>46060.64861111111</v>
       </c>
-      <c r="B39" s="74" t="n">
+      <c r="B39" s="75" t="n">
         <v>83.06999999999999</v>
       </c>
-      <c r="C39" s="75" t="inlineStr">
+      <c r="C39" s="76" t="inlineStr">
         <is>
           <t>composição incompleta: só peso, sem bioimpedância</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="73" t="n">
+      <c r="A40" s="74" t="n">
         <v>46083.51041666666</v>
       </c>
-      <c r="B40" s="74" t="n">
+      <c r="B40" s="75" t="n">
         <v>81.98</v>
       </c>
-      <c r="C40" s="75" t="inlineStr">
+      <c r="C40" s="76" t="inlineStr">
         <is>
           <t>composição incompleta: só peso, sem bioimpedância</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="73" t="n">
+      <c r="A41" s="74" t="n">
         <v>46106.50208333333</v>
       </c>
-      <c r="B41" s="74" t="n">
+      <c r="B41" s="75" t="n">
         <v>81.03</v>
       </c>
-      <c r="C41" s="75" t="inlineStr">
+      <c r="C41" s="76" t="inlineStr">
         <is>
           <t>composição incompleta: só peso, sem bioimpedância</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="73" t="n">
+      <c r="A42" s="74" t="n">
         <v>46129.51666666667</v>
       </c>
-      <c r="B42" s="74" t="n">
+      <c r="B42" s="75" t="n">
         <v>79.92</v>
       </c>
-      <c r="C42" s="75" t="inlineStr">
+      <c r="C42" s="76" t="inlineStr">
         <is>
           <t>composição incompleta: só peso, sem bioimpedância</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="73" t="n">
+      <c r="A43" s="74" t="n">
         <v>46152.65833333333</v>
       </c>
-      <c r="B43" s="74" t="n">
+      <c r="B43" s="75" t="n">
         <v>78.62</v>
       </c>
-      <c r="C43" s="75" t="inlineStr">
+      <c r="C43" s="76" t="inlineStr">
         <is>
           <t>composição incompleta: só peso, sem bioimpedância</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="73" t="n">
+      <c r="A44" s="74" t="n">
         <v>46175.50138888889</v>
       </c>
-      <c r="B44" s="74" t="n">
+      <c r="B44" s="75" t="n">
         <v>77.26000000000001</v>
       </c>
-      <c r="C44" s="75" t="inlineStr">
+      <c r="C44" s="76" t="inlineStr">
         <is>
           <t>composição incompleta: só peso, sem bioimpedância</t>
         </is>

</xml_diff>

<commit_message>
README: imagens e exemplo fictício atualizados (versão 2.1.0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exemplo/exemplo-transformacao.xlsx
+++ b/docs/exemplo/exemplo-transformacao.xlsx
@@ -2314,7 +2314,7 @@
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="2">
-        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"/"&amp;YEAR(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0)))&amp;" às "&amp;RIGHT("0"&amp;HOUR(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 12:56"</f>
+        <f>"Última leitura: "&amp;RIGHT("0"&amp;DAY(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"/"&amp;RIGHT("0"&amp;MONTH(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"/"&amp;YEAR(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0)))&amp;" às "&amp;RIGHT("0"&amp;HOUR(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;":"&amp;RIGHT("0"&amp;MINUTE(INDEX('Medições Corporais'!$A$4:$A$147,MATCH(MAX('Medições Corporais'!$R$4:$R$147),'Medições Corporais'!$R$4:$R$147,0))),2)&amp;"  ·  "&amp;COUNT('Medições Corporais'!$A$4:$A$147)&amp;" leituras aceites  ·  Atualizado em 11/10/2026 16:40"</f>
         <v/>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:56</t>
+          <t>Atualizado em 11/10/2026 16:40</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:56</t>
+          <t>Atualizado em 11/10/2026 16:40</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6299,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>144 leituras aceites · Atualizado em 11/10/2026 12:56 · fórmulas: massa gorda e médias móveis de 7 dias</t>
+          <t>144 leituras aceites · Atualizado em 11/10/2026 16:40 · fórmulas: massa gorda e médias móveis de 7 dias</t>
         </is>
       </c>
     </row>
@@ -15221,7 +15221,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>Atualizado em 11/10/2026 12:56</t>
+          <t>Atualizado em 11/10/2026 16:40</t>
         </is>
       </c>
     </row>

</xml_diff>